<commit_message>
Updated Message Scam Detector
</commit_message>
<xml_diff>
--- a/services/message_detector/outputs/ScamSense_Batch_Message_Analysis.xlsx
+++ b/services/message_detector/outputs/ScamSense_Batch_Message_Analysis.xlsx
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -44,11 +41,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001565C0"/>
+        <fgColor rgb="006C3BFF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -56,22 +53,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -461,379 +449,377 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Predicted Scam Type</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Confidence Score (ML Model)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Confidence Level (ML Model Certainty)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Confidence Gap (Top 1 vs Top 2 Model Prediction Score Difference)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Risk Level (Final ScamSense Assessment)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Cross-Verification (Model Agreement)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>AI Summary</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Why Suspicious / Legitimate Explanation</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Scam Indicators</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Safety Advice</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Recommended Actions</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Prevention Tips</t>
         </is>
       </c>
     </row>
     <row r="2" ht="300" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Dear Customer, your DBS bank account has been temporarily suspended due to unusual activity. Verify your account immediately at https://secure-dbs-verify-login.com to avoid permanent suspension.</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Banking Scam</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>99.88%</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>99.84%</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>No - Not required</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>This message appears likely to be a banking scam. It uses common tactics to create urgency and direct you to a fake website, aiming to trick you into revealing sensitive banking information.</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>The message claims your DBS bank account has been 'temporarily suspended due to unusual activity' and demands 'immediate' verification to prevent 'permanent suspension'. This creates a false sense of urgency, a common characteristic of banking scams, which impersonate legitimate institutions to pressure individuals. The inclusion of a suspicious link, 'https://secure-dbs-verify-login.com', which is not an official DBS domain, is a strong indicator of a phishing attempt. The original machine learning model identified keywords like 'account', 'bank', 'unusual', and 'immediately' as top contributors to its high-confidence prediction of a Banking Scam, which aligns with the final ScamSense assessment.</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>1. **Unexpected Account Suspension Claim**: The message states your DBS bank account has been 'temporarily suspended due to unusual activity,' which is a common tactic used by scammers to alarm recipients, consistent with 'Unexpected messages claiming that a bank account has been suspended or compromised.'
-2. **Urgent Call to Action**: It demands you 'Verify your account immediately... to avoid permanent suspension.' This creates an urgent deadline that discourages careful verification, a key warning sign.
-3. **Suspicious Website Link**: The link provided, 'https://secure-dbs-verify-login.com', is not a legitimate DBS website. Scammers often use slightly altered or unfamiliar domain names to trick users into entering login credentials on fake sites.
-4. **Request for Immediate Login/Verification**: The link is designed to prompt you to log in or 'verify' your account, which is a typical victim request in banking scams aiming to steal online banking usernames and passwords.</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>1. Always be suspicious of unexpected messages, especially those claiming urgent issues with your bank account.
-2. Never click on links in suspicious SMS messages or emails, even if they appear to be from a known sender.
-3. Be cautious of any communication that pressures you to take immediate action, particularly if it involves your financial accounts.</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>1. Do not click on the link provided in the message or respond to the sender.
-2. Contact DBS directly using their official customer service hotline or through their official website/app to verify any account-related concerns.
-3. If you accidentally clicked the link or provided any information, immediately contact your bank to secure your account and monitor for unauthorised transactions.
-4. Consider reporting this suspicious message to ScamShield or the relevant authorities.</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>1. Always access your online banking services through official banking applications or by typing the bank's official website address directly into your browser.
-2. Never share your passwords, PINs, or One-Time Passwords (OTPs) with anyone, regardless of who they claim to be.
-3. Enable multi-factor authentication and banking transaction notifications for all your bank accounts to enhance security.
-4. Regularly review your bank account activity for any unauthorised transactions and keep your mobile devices and banking applications updated with the latest security patches.</t>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>This message appears highly likely to be a Banking Scam. It uses tactics common in financial fraud, such as creating urgency around an account suspension and directing you to a suspicious link for 'verification'. The high confidence level reflects the strong indicators of a scam present in the message.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>The message employs classic banking scam tactics by creating a false sense of urgency and fear regarding an account suspension, demanding 'immediate' action to avoid 'permanent suspension'. It then directs the recipient to a highly suspicious and unofficial website link (secure-dbs-verify-login.com) to 'verify' their account. This is a common method used by scammers to phish for login credentials and sensitive financial information, aligning with the retrieved knowledge on banking scams that impersonate financial institutions and use fake websites.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>1. The message contains an unexpected notification about a bank account (DBS) being 'temporarily suspended due to unusual activity', which is a common tactic used by scammers to cause alarm.
+2. It includes a strong sense of urgency, urging the user to 'Verify your account immediately' to 'avoid permanent suspension', pressuring them into hasty action without careful verification.
+3. The message provides a suspicious URL, 'https://secure-dbs-verify-login.com', which attempts to mimic an official bank domain but is clearly not the legitimate DBS website, indicating a phishing attempt designed to steal login credentials.
+4. The request to 'verify your account' by clicking an unsolicited link is a typical method used by criminals to trick individuals into revealing sensitive information.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>1. Treat any unexpected message claiming issues with your bank account with extreme caution. Do not trust messages that pressure you to take immediate action through provided links.
+2. Always verify the legitimacy of such claims directly with your bank by contacting them through their official hotline number (found on their official website or bank card) or by logging into your account via their official mobile app or website, not through links in suspicious messages.
+3. Never share your passwords, PINs, One-Time Passwords (OTPs), or any other sensitive banking credentials in response to unsolicited messages or calls.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>1. Do not click on the provided link or any other links within this message.
+2. Do not reply to the sender or attempt to communicate with them.
+3. Contact DBS Bank immediately using their official customer service channels (not numbers or links from the message) to confirm the status of your account.
+4. Preserve the message by taking a screenshot or forwarding it to official scam reporting platforms like ScamShield, if available in your region.
+5. Monitor your official bank account statements closely for any unusual or unauthorised transactions.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>1. Always access your online banking services by typing the bank's official website address directly into your browser or using their official mobile application.
+2. Be highly suspicious of any unsolicited messages, emails, or calls that create a sense of urgency, threaten account closure, or ask for immediate action to 'verify' your account.
+3. Enable multi-factor authentication (MFA) on all your banking and online accounts for an added layer of security.
+4. Regularly review your bank account activity and transaction notifications for any irregularities and report them promptly to your bank.
+5. Learn to identify common phishing signs, such as unofficial-looking sender addresses, poor grammar, and suspicious URLs, even if they appear to resemble legitimate bank names.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="300" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Congratulations! You have been selected for a remote data entry position earning SGD 5,000 per month. No experience is required. Register now at https://easy-work-from-home-jobs.net to secure your position.</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Job Scam</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>91.14%</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>87.64%</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>No - Not required</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>This message appears likely to be a Job Scam with a high risk. It presents an unsolicited offer for a remote data entry position with an unusually high salary and no experience required, which are common characteristics of fraudulent recruitment schemes designed to lure unsuspecting job seekers.</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>The message exhibits several characteristics commonly associated with job scams. It starts with an immediate 'Congratulations!' for an unsolicited job offer, promising a high salary of 'SGD 5,000 per month' for a 'remote data entry position' with 'No experience required'. Such offers of high income for minimal effort or experience are typical lures in job scams. The call to 'Register now at https://easy-work-from-home-jobs.net to secure your position' creates urgency and directs to a generic-sounding website, often a tactic to collect personal information or induce payments. These elements are consistent with common scam tactics identified by the ScamSense system and our retrieved scam knowledge, which highlights fake recruitment, unrealistic salaries, and requests for upfront actions like registration on unverified platforms. The AI model's contributing keywords like 'position', 'remote', 'experience', 'register', and 'congratulations' further underscore these suspicious aspects.</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>1. Unsolicited job offer with immediate 'Congratulations!' without any application process.
-2. Promise of an unusually high income (SGD 5,000 per month) for a minimal-skill 'data entry position'.
-3. Requirement of 'No experience' for a high-paying role, a common tactic to appeal to a wide range of victims.
-4. Urgent call to action ('Register now') on a generic-sounding website (easy-work-from-home-jobs.net), which may not be a legitimate company portal.
-5. The offer of a 'remote' position, frequently exploited by scammers to target individuals seeking flexible work.</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>1. Be highly suspicious of any unsolicited job offers, especially those promising high pay for little effort or experience.
-2. Never click on links or register on websites provided in suspicious or unexpected job offers.
-3. Legitimate employers typically do not offer jobs without a formal interview process or require upfront payments.
-4. Always verify job opportunities and company details through official, independent sources, not just the information provided in the message.</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>1. Do not click on the link provided in the message.
-2. Do not register or provide any personal or financial information on the website mentioned.
-3. Block the sender of this message to prevent further scam attempts.
-4. Report this message as a scam to relevant authorities, such as the Singapore Police Force (SPF) via their anti-scam hotline or the ScamShield app.</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>1. Verify job advertisements and company legitimacy through official websites or recognised recruitment platforms before applying or responding to offers.
-2. Exercise caution with job offers that promise unusually high income for minimal work or experience.
-3. Never pay any fees (e.g., for registration, training, equipment, or administrative costs) to secure an employment opportunity.
-4. Research the employer and confirm the recruiter's identity using official company contact information, not just what's provided in the message.
-5. Be wary of employers who avoid formal interviews or insist on communicating only through messaging applications rather than official channels.</t>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>The message you received appears likely to be a job scam, carrying a high risk. It shows characteristics commonly associated with fraudulent employment offers, such as an unsolicited 'congratulations' for a high-paying remote role with no experience required, and a prompt to register on an unfamiliar website.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>This message is highly suspicious because it uses several tactics common in job scams. It starts with an unsolicited 'Congratulations!' for a job you didn't apply for, offering an unusually high salary of SGD 5,000 per month for a 'remote data entry position' with 'No experience required'. Such offers often aim to entice victims with unrealistic promises of easy money, as highlighted by ScamSense's retrieved knowledge. The immediate request to 'Register now' at an unknown URL without any formal interview process is another strong red flag, as legitimate companies typically follow a more structured recruitment process and use official channels. These elements, including 'position', 'remote', 'experience', 'register', and 'congratulations', were also key factors in the machine learning model's assessment.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>1. Unsolicited 'Congratulations!' for a job you didn't apply for, which is a common tactic used by scammers to create a false sense of urgency and legitimacy (KNOWLEDGE RESULT 3).
+2. Promise of an unusually high salary (SGD 5,000/month) for a 'remote data entry position' requiring 'No experience', which are unrealistic offers designed to attract victims, often seen in job scams (KNOWLEDGE RESULT 2, 3, 4).
+3. Immediate selection for a 'position' without any formal application, interview, or assessment process (KNOWLEDGE RESULT 3).
+4. Instruction to 'Register now' at an unfamiliar external website (easy-work-from-home-jobs.net), which may be a phishing attempt or lead to requests for personal information or upfront payments (KNOWLEDGE RESULT 5).
+5. The offer of a 'remote' and 'flexible' employment opportunity, which are frequently exploited by scammers to target individuals seeking such arrangements (KNOWLEDGE RESULT 1, 3).</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>1. Always be suspicious of unsolicited job offers, especially those promising high pay for minimal effort or experience, as these are common characteristics of job scams.
+2. Never click on suspicious links in unexpected messages, as they could lead to malicious websites designed to steal your information or install harmful software.
+3. Do not provide personal or financial information, such as bank account details or identification documents, to unverified sources or through unsecured websites.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>1. Do not click on the provided link or attempt to register on the website.
+2. Block the sender's number or email address to prevent further suspicious communications.
+3. Report the message to your telecommunications provider or the Singapore Police Force via their Anti-Scam Hotline at 1800-722-6688 or online at www.scamalert.sg.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>1. Verify job advertisements and company legitimacy through official company websites or recognised recruitment platforms before applying or engaging with any offer (KNOWLEDGE RESULT 2).
+2. Be wary of any job offer that asks you to pay fees for training, registration, work permits, or equipment, as legitimate employers generally do not request upfront payments from job applicants (KNOWLEDGE RESULT 2, 3, 5).
+3. Legitimate employers typically conduct formal interviews and provide written employment contracts through official communication channels (KNOWLEDGE RESULT 2).
+4. Research the company and confirm recruiter identities using official contact information before accepting any job offer or sharing personal details (KNOWLEDGE RESULT 2).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="300" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Your parcel delivery was unsuccessful because the shipping address is incomplete. Please pay a redelivery fee of SGD 2.99 at https://sgparcel-redelivery.com within 24 hours to receive your package.</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Parcel Scam</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>No - Not required</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>The message you received appears likely to be a parcel scam, which commonly exploits online shopping and delivery processes to trick individuals into making payments or revealing personal information.</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>This message shows several characteristics highly associated with parcel scams. It claims an unsuccessful delivery due to an 'incomplete address,' a frequent tactic used by scammers to create a fabricated problem that requires immediate user action. The request for a redelivery fee of SGD 2.99 is typical, as scammers often ask for small amounts to reduce suspicion and encourage quick payment. Crucially, the message includes a suspicious link, 'https://sgparcel-redelivery.com,' which is designed to mimic an official site but is likely a phishing page. Furthermore, the imposed 24-hour deadline creates a false sense of urgency, pressuring you to act without independently verifying the notification.</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>1. Unexpected notification of an unsuccessful parcel delivery due to an 'incomplete address'.
-2. Request for a redelivery fee (SGD 2.99) via a provided link.
-3. Inclusion of a suspicious or unofficial-looking website link ('https://sgparcel-redelivery.com') for payment.
-4. A short deadline ('within 24 hours') to complete the payment, creating a false sense of urgency.</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>1. Do not click on the provided link, as it likely leads to a fraudulent website designed to steal your payment details, personal information, or install malware.
-2. Always verify unexpected delivery notifications directly with the courier company through their official website or mobile application, which you access independently.
-3. Be extremely cautious of requests for unexpected payments, especially for 'redelivery fees' or 'customs duties,' as these are common tactics in parcel scams.</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>1. Ignore and delete this suspicious message to avoid any accidental interaction with the scammers.
-2. Preserve the message (e.g., by taking a screenshot) as evidence if you intend to report it to authorities.
-3. Report suspicious messages like this one to relevant local authorities, such as through the ScamShield app if you are in Singapore.
-4. Contact your bank immediately if you have already clicked the link or submitted any payment information or personal details.</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>1. Only track parcels and manage deliveries through the courier company's official website or mobile application, which you access by typing the URL yourself or using a trusted app.
-2. Verify any unexpected delivery notifications by checking your recent purchases and expected deliveries directly with the sender or retailer.
-3. Never provide passwords, One-Time Passwords (OTPs), or banking credentials through links contained in unsolicited delivery messages.
-4. Be highly suspicious of messages demanding immediate payment for customs duties, taxes, or redelivery fees for parcels you were not expecting or have not verified.</t>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>The message you received appears likely to be a parcel scam, classified with a high risk and high confidence. It exhibits common characteristics of fraudulent delivery notifications, attempting to trick you into paying a redelivery fee through a suspicious link.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>This message shows strong characteristics associated with a parcel scam. It claims your 'parcel delivery was unsuccessful' due to an 'incomplete shipping address' and demands a 'redelivery fee' of SGD 2.99, creating an urgent situation with a '24 hours' deadline. The message then directs you to a non-official-looking website, 'https://sgparcel-redelivery.com', to make this payment. These elements, particularly the unexpected fee and suspicious link, are key indicators of a scam designed to exploit routine delivery expectations, aligning with keywords like 'delivery', 'package', 'parcel', and 'shipping' that influenced the initial analysis.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>1. An unexpected notification claiming 'parcel delivery was unsuccessful' due to an 'incomplete shipping address'.
+2. A demand for a 'redelivery fee' (SGD 2.99), which legitimate courier services typically handle through official procedures, not urgent external links.
+3. The presence of a suspicious URL, 'https://sgparcel-redelivery.com', which does not appear to be an official courier website, indicating a potential phishing attempt.
+4. A sense of urgency, requiring payment 'within 24 hours', a common tactic used by scammers to pressure victims into acting quickly without verification.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>1. Do not click on the provided link or any links in suspicious delivery messages.
+2. Never provide personal, banking, or credit card details on websites accessed through unsolicited links.
+3. Legitimate courier companies do not typically request urgent payments for redelivery via unverified links. Always verify delivery notifications directly with the sender or courier using their official contact channels (e.g., their official website or app).</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>1. Ignore and immediately delete this suspicious message to prevent accidental clicks.
+2. If you are expecting a parcel, verify its status directly through the courier's official website or app by entering your tracking number manually.
+3. Preserve the SMS message or email as evidence by taking a screenshot if you believe you have been targeted by a scam.
+4. Report this suspicious message to the authorities, such as through the ScamShield app or the Singapore Police Force if any financial loss has occurred.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>1. Always verify parcel notifications by checking your recent purchases and expected deliveries against official tracking information.
+2. Track parcels only through the courier company's official website or mobile application, never through links in unexpected messages.
+3. Be highly cautious of any requests for unexpected delivery fees, customs duties, or taxes, especially if they demand immediate payment.
+4. Carefully inspect website addresses before entering any personal or payment information; look for official domain names and secure connections (https).
+5. Never provide passwords, One-Time Passwords (OTPs), or banking credentials via delivery websites or unexpected links.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="300" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>SingPost is delivering your parcel CNSGS005229637 by today. Please ensure someone is available to receive it. If you are not at home, it will be delivered to a safe place near your doorstep.</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Legitimate</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>48.88%</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>25.48%</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Yes - 3/4 models agreed (75.00%)</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>The ScamSense system assessed your message as appearing likely to be legitimate, indicating a low risk. This assessment is supported by internal verification, though the overall confidence in this classification is low.</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>The message appears legitimate because it follows a standard delivery notification format from SingPost, provides a parcel reference number (CNSGS005229637), and describes common delivery procedures such as ensuring availability and delivery to a safe place if not at home. It does not contain requests for payment, sensitive personal information, or suspicious links commonly associated with parcel scams, which are characteristics of genuine communications. Keywords like 'parcel', 'home', 'available', 'delivered', and 'ensure' also align with typical delivery updates.</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>The message appears likely to be a legitimate delivery notification from SingPost based on the available evidence and its consistent format.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>The message appears legitimate because it uses common language associated with genuine parcel deliveries, mentioning keywords such as 'parcel', 'home', 'available', 'delivered', and 'ensure'. It follows a normal service-notification format from a known courier (SingPost) and provides standard delivery information without significant requests for money, sensitive credentials, unusual urgency, or suspicious links commonly associated with scams.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>No scam indicators were identified because this message appears likely to be legitimate.</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>1. Even though this message appears legitimate, always exercise caution if you did not expect a delivery or if the message seems out of place.
-2. Verify the delivery status directly through SingPost's official website or app using the provided tracking number, rather than relying solely on the message.</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>1. Verify the delivery status of parcel CNSGS005229637 directly on the official SingPost website or app, especially if you did not anticipate a delivery.
-2. If the message had included links, avoid clicking on them and instead navigate to the official courier website manually.
-3. Do not provide personal or financial details in response to unexpected delivery messages.</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>1. Track parcels only through the courier company's official website or mobile application.
-2. Be cautious of requests for unexpected delivery fees or personal information.
-3. If you receive an unexpected delivery notification, confirm it with the sender or retailer before taking any action.
-4. Avoid clicking links contained in unsolicited delivery messages.</t>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1. Always verify unexpected delivery notifications through official channels, especially if you did not anticipate a parcel. Even if a message appears legitimate, confirm its authenticity, particularly if it asks for personal details or actions beyond what is standard for a delivery.
+2. Be cautious if you did not initiate the activity or are not expecting a parcel with the stated tracking number. Cross-reference the information with your recent purchases and expected deliveries.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>1. If you are expecting a parcel, cross-reference the tracking number (CNSGS005229637) with your order details on the official SingPost website or app.
+2. If you are not expecting a parcel, consider deleting the message after independent verification through official SingPost channels, not through any links in the message.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>1. Track parcels only through the courier company's official website or mobile application, not via links in unsolicited messages.
+2. Avoid clicking links contained in unexpected delivery messages; always navigate directly to official websites.
+3. Confirm unexpected delivery notifications with the sender or retailer directly if you are unsure of their legitimacy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated Message Scam Detector UI
</commit_message>
<xml_diff>
--- a/services/message_detector/outputs/ScamSense_Batch_Message_Analysis.xlsx
+++ b/services/message_detector/outputs/ScamSense_Batch_Message_Analysis.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$M$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -553,279 +553,48 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>The message you received, claiming your DBS bank account has been temporarily suspended due to unusual activity and requesting immediate verification via a link, appears highly likely to be a banking scam. This assessment is made with high confidence due to the presence of several common scam characteristics.</t>
+          <t>The message you received appears highly likely to be a Banking Scam. It shows characteristics commonly used by criminals to trick individuals into revealing sensitive financial information, posing a high risk to your financial security.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>This message exhibits classic warning signs of a banking scam. It creates a false sense of urgency by stating your 'DBS bank account has been temporarily suspended' and demanding you 'verify your account immediately' to 'avoid permanent suspension'. This tactic is used to pressure you into acting without careful verification. The message also includes a suspicious link, 'https://secure-dbs-verify-login.com', which is designed to mimic an official bank website but is not the legitimate DBS domain. Scammers often use such fake websites to steal your login credentials or other sensitive information. The original machine learning model identified keywords like 'account', 'bank', 'unusual', and 'immediately' as strong indicators of this scam type.</t>
+          <t>The message claims your DBS bank account has been 'temporarily suspended due to unusual activity' and urges you to 'verify your account immediately' via a provided link. This creates a false sense of urgency and directs you to a suspicious URL (secure-dbs-verify-login.com) that is not the official DBS website. These are classic tactics used in banking scams to phish for your login credentials.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>1. The message creates a false sense of urgency by claiming immediate action is required to prevent 'permanent suspension' of your 'DBS bank account'.
-2. It refers to 'unusual activity' as a reason for suspension, a common scam narrative to create alarm.
-3. The provided URL, 'https://secure-dbs-verify-login.com', is not an official DBS website and is designed to trick users into revealing sensitive information on a fraudulent site.
-4. The request to 'verify your account immediately' is a typical tactic to pressure victims into making hasty decisions and clicking malicious links.</t>
+          <t>1. The message creates a false sense of urgency by claiming 'unusual activity' and threatening 'permanent suspension' of your account if immediate action is not taken.
+2. It includes a suspicious link (https://secure-dbs-verify-login.com) that impersonates the bank's name but is not the official bank website, which is a common characteristic of phishing attempts.
+3. The language demands 'immediate' verification, discouraging careful consideration and verification through official channels.
+4. Keywords like 'account', 'bank', 'unusual', and 'immediately' were identified as top contributors by our analysis, aligning with common patterns in banking scams.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>1. Do not click on any links provided in suspicious messages, especially those claiming account issues or requiring immediate verification.
-2. Never enter your banking login credentials, One-Time Passwords (OTPs), or other personal financial information into websites accessed via unsolicited links.
-3. Always be suspicious of unexpected messages that demand immediate action or warn of severe consequences like account suspension.</t>
+          <t>1. Do NOT click on any links provided in unexpected messages, especially those claiming to be from your bank.
+2. Never enter your banking login credentials, PINs, or One-Time Passwords (OTPs) into websites accessed via unsolicited links.
+3. Always contact your bank directly using their official contact information (found on their official website or the back of your card) to verify any suspicious messages or account alerts.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>1. Stop all communication with the sender of this message immediately.
-2. Contact DBS directly using the official customer service number found on their official website or the back of your bank card, not any number provided in the suspicious message, to verify the status of your account.
-3. Do not provide any personal, financial, or login details to anyone who contacts you unexpectedly, regardless of who they claim to be.
-4. Preserve the message as evidence (e.g., by taking a screenshot) and report it to relevant authorities like ScamShield if applicable.
-5. Monitor your bank accounts closely for any unauthorised transactions.</t>
+2. Contact DBS Bank directly via their official customer service hotline to inquire about your account status if you have genuine concerns.
+3. Do not provide any personal, financial, or login information to the sender or through the provided link.
+4. Delete the suspicious message to avoid accidentally interacting with it in the future.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>1. Always access online banking services only through official banking applications or by typing the bank's official website address directly into your browser.
-2. Never share your passwords, PINs, or OTPs with anyone, even if they claim to be from your bank.
-3. Verify any suspicious messages or calls by contacting your bank through their official customer service channels, which you find independently.
-4. Carefully inspect the full website address (URL) before entering any login credentials; legitimate banking websites will have secure and familiar domain names.
-5. Enable multi-factor authentication (MFA) and banking transaction notifications on your accounts for an added layer of security.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="300" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Congratulations! You have been selected for a remote data entry position earning SGD 5,000 per month. No experience is required. Register now at https://easy-work-from-home-jobs.net to secure your position.</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Job Scam</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>91.14%</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>87.64%</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>No - Not required</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>This message appears highly likely to be a Job Scam, characterized by an unsolicited offer for a high-paying remote position with no experience required, directing you to register on an unfamiliar website.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>The message exhibits several common characteristics of job scams, including an unsolicited "congratulations" for an immediate job offer. It promises an unusually high salary (SGD 5,000 per month) for a "remote data entry position" that requires "No experience," which is a classic tactic to lure victims. The instruction to "Register now" on a suspicious-looking domain (https://easy-work-from-home-jobs.net) is a strong indicator of a fraudulent attempt to collect personal information, request payments, or lead to malicious activities. These elements align with common scam tactics described in our knowledge base, such as advertising fake job vacancies with unrealistic salaries and contacting individuals without a formal application process. The analysis by our AI model highlighted keywords like 'position', 'remote', 'experience', 'register', and 'congratulations' as contributing to this assessment.</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>1. Unsolicited job offer with a 'Congratulations' for immediate selection, bypassing a formal application process.
-2. Promise of unusually high income (SGD 5,000 per month) for a simple 'remote data entry position' with 'No experience is required'.
-3. Directing the user to 'Register now' on a generic and suspicious-looking domain (https://easy-work-from-home-jobs.net) rather than an official company website.</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>1. Always be skeptical of unsolicited job offers, especially those promising high pay for minimal effort or experience.
-2. Verify any job opportunity through the company's official website or recognised recruitment platforms before providing personal information or clicking on links.
-3. Legitimate employers do not typically offer jobs immediately without interviews or a proper assessment process.</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>1. Do not click on the link provided in the message or attempt to register on the website.
-2. Do not reply to the message or engage with the sender in any way.
-3. Block the sender's number or email address to prevent further unsolicited communication.
-4. Report the message to your telecommunications provider or relevant authorities (e.g., Singapore Police Force if in Singapore).</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>1. Verify all job advertisements through official channels, such as company websites or established job portals.
-2. Be extremely cautious of job offers that guarantee high income for minimal work or no experience.
-3. Never make any payments for job applications, training, work permits, or equipment purchases.
-4. Thoroughly research the employer and the recruiter's identity before sharing any personal or financial information.
-5. Avoid sharing sensitive personal details like bank account information or identification documents unless the employer has been fully verified through official means.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="300" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Your parcel delivery was unsuccessful because the shipping address is incomplete. Please pay a redelivery fee of SGD 2.99 at https://sgparcel-redelivery.com within 24 hours to receive your package.</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Parcel Scam</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>No - Not required</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>The message you received appears likely to be a parcel scam, which is a high-risk type of fraud. ScamSense AI has assessed this with high confidence, indicating it shows strong characteristics of attempts to trick individuals into paying fake redelivery fees or revealing personal information under the guise of an undeliverable package.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>This message is highly suspicious because it claims an 'unsuccessful delivery' due to an 'incomplete shipping address' and demands a 'redelivery fee' of SGD 2.99. Scammers frequently use such tactics, as highlighted in our scam knowledge, to create urgency and a seemingly legitimate reason for a small payment. The message also includes a suspicious URL (sgparcel-redelivery.com) which is unlikely to be an official courier website, and imposes a short deadline ('within 24 hours') to pressure you into acting quickly without proper verification. These elements are consistent with common parcel scam patterns described in our intelligence, where victims are directed to fake websites for payment.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>1. An unsolicited message claiming an 'unsuccessful delivery' due to an 'incomplete shipping address', a common tactic to initiate a scam.
-2. A demand for an unexpected 'redelivery fee' (SGD 2.99), which is often a small amount designed to lower suspicion and encourage quick payment.
-3. The presence of a suspicious, unofficial-looking URL (https://sgparcel-redelivery.com) for payment, which is a strong indicator of a phishing attempt.
-4. A sense of urgency created by a deadline ('within 24 hours') to pressure the recipient into immediate action without proper verification.</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>1. Do not click on any links in the message, especially the payment link, as it may lead to a phishing website designed to steal your personal or financial information.
-2. Never provide personal, banking, or credit card details in response to unexpected delivery notifications, especially if they come from unknown or suspicious sources.
-3. Always verify the status of any parcel directly through the courier company's official website or mobile application, using a tracking number you initiated or received from a trusted sender.</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>1. Immediately ignore and delete this suspicious message to prevent accidental clicks or engagement.
-2. If you have clicked the link or submitted any payment information, contact your bank or credit card company immediately to report potential fraud and monitor your accounts for suspicious activity.
-3. Preserve a screenshot of the message as evidence before deleting it, in case it's needed for reporting purposes.
-4. Report the message to the relevant authorities, such as ScamShield or the Singapore Police Force, especially if any financial loss has occurred or personal information was compromised.</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>1. Be vigilant about unexpected delivery notifications, especially if you are not anticipating a package or if the sender is unfamiliar.
-2. Only track parcels or make payments through the courier company's official website or mobile application, accessed by typing the URL directly into your browser or using a trusted app.
-3. Carefully inspect website addresses (URLs) for legitimacy before entering any personal or payment information; look for discrepancies in official company names and domain names.
-4. Be cautious of requests for unexpected delivery or customs fees, particularly if they come with a sense of urgency or via suspicious links rather than established procedures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="300" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>SingPost is delivering your parcel CNSGS005229637 by today. Please ensure someone is available to receive it. If you are not at home, it will be delivered to a safe place near your doorstep.</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Legitimate</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>48.88%</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>25.48%</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Yes - 3/4 models agreed (75.00%)</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Based on the analysis, the message appears likely to be a legitimate delivery notification from SingPost. Internal verification also supports this assessment, with 3 out of 4 models agreeing with this classification. However, a low confidence level suggests that caution is still advisable, especially if you were not expecting a parcel.</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>The message appears legitimate because it uses a standard delivery notification format, mentioning a specific courier (SingPost) and parcel tracking number. It provides clear instructions about receiving the parcel ('ensure someone is available') and an alternative delivery method ('delivered to a safe place near your doorstep') which is consistent with normal courier service practices. The language used is direct and does not contain unusual urgency, requests for sensitive personal information, or suspicious links, which are common characteristics of parcel scams.</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>No scam indicators were identified because this message appears likely to be legitimate.</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>1. Even though this message appears legitimate, it's always safest to verify any unexpected delivery notifications. If you were not expecting a parcel, consider checking your recent online purchases or tracking your deliveries directly through the official SingPost website or app, using the provided tracking number.
-2. Be cautious of any follow-up messages that might ask you to click on links, provide personal details, or pay unexpected fees for redelivery, as these could be attempts to exploit an otherwise legitimate-looking notification.</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>1. If you are expecting a parcel with this tracking number, you can track it via the official SingPost website or mobile application.
-2. If you are unsure or did not expect a parcel, refrain from clicking any links in future messages related to this delivery. Instead, visit the official SingPost website directly to check on the parcel's status or contact their customer service if needed.
-3. Monitor your bank and online accounts for any suspicious activity, especially if you encounter similar messages that request personal or payment information.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>1. Always verify delivery notifications by checking your recent purchases and expected deliveries directly through the retailer or courier's official channels.
-2. Track parcels only through the courier company's official website or mobile application, avoiding links in unsolicited messages.
-3. Never provide passwords, One-Time Passwords (OTPs), or banking credentials through delivery websites unless you have independently verified the request and the website's authenticity.
-4. Be cautious of requests for unexpected delivery fees or customs duties, and always confirm these through official sources before making any payment.</t>
+          <t>1. Access your online banking services only through the official banking application or by typing the bank's official website address directly into your browser.
+2. Be wary of any unsolicited messages or calls that request your passwords, PINs, or OTPs, as legitimate banks will never ask for these details in such a manner.
+3. Enable multi-factor authentication (MFA) on all your banking and online accounts for an added layer of security.
+4. Regularly review your bank statements and account activity for any unauthorized transactions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M5"/>
+  <autoFilter ref="A1:M2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Message Scan and Shared Chatbot for Message Scan
</commit_message>
<xml_diff>
--- a/services/message_detector/outputs/ScamSense_Batch_Message_Analysis.xlsx
+++ b/services/message_detector/outputs/ScamSense_Batch_Message_Analysis.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$M$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -553,48 +553,278 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>The message you received appears highly likely to be a Banking Scam. It shows characteristics commonly used by criminals to trick individuals into revealing sensitive financial information, posing a high risk to your financial security.</t>
+          <t>This message appears highly likely to be a banking scam. It employs tactics commonly used by fraudsters to deceive individuals into revealing sensitive financial information or login credentials by creating a false sense of urgency regarding an account suspension.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>The message claims your DBS bank account has been 'temporarily suspended due to unusual activity' and urges you to 'verify your account immediately' via a provided link. This creates a false sense of urgency and directs you to a suspicious URL (secure-dbs-verify-login.com) that is not the official DBS website. These are classic tactics used in banking scams to phish for your login credentials.</t>
+          <t>The message is highly suspicious because it uses common scam tactics: it claims your bank account has been suspended due to 'unusual activity' to create alarm, and then demands immediate action by directing you to a non-official, suspicious website to 'verify' your account. This strategy is designed to trick you into entering your banking details on a fraudulent site.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>1. The message creates a false sense of urgency by claiming 'unusual activity' and threatening 'permanent suspension' of your account if immediate action is not taken.
-2. It includes a suspicious link (https://secure-dbs-verify-login.com) that impersonates the bank's name but is not the official bank website, which is a common characteristic of phishing attempts.
-3. The language demands 'immediate' verification, discouraging careful consideration and verification through official channels.
-4. Keywords like 'account', 'bank', 'unusual', and 'immediately' were identified as top contributors by our analysis, aligning with common patterns in banking scams.</t>
+          <t>1. An unsolicited message claiming your bank account has been temporarily suspended due to 'unusual activity,' which is a common scare tactic used by scammers to create panic.
+2. The demand for immediate action to 'verify your account' at a provided link to avoid 'permanent suspension,' which is a classic urgency tactic to prevent careful verification.
+3. The presence of a suspicious URL (secure-dbs-verify-login.com) that attempts to mimic a legitimate bank website but is not the official DBS domain, strongly indicating a phishing attempt.
+4. Keywords such as 'account,' 'bank,' 'unusual,' and 'immediately' in the message were identified as significant contributors to the scam classification, reflecting patterns in fraudulent communications.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>1. Do NOT click on any links provided in unexpected messages, especially those claiming to be from your bank.
-2. Never enter your banking login credentials, PINs, or One-Time Passwords (OTPs) into websites accessed via unsolicited links.
-3. Always contact your bank directly using their official contact information (found on their official website or the back of your card) to verify any suspicious messages or account alerts.</t>
+          <t>1. Always be suspicious of unexpected messages claiming issues with your bank account, especially those that demand immediate action or contain unusual links.
+2. Never click on links in suspicious messages. Banks will typically not ask you to verify your account or login via a link in an SMS or email.
+3. Do not share your online banking passwords, PINs, or One-Time Passwords (OTPs) with anyone, regardless of who they claim to be.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>1. Stop all communication with the sender of this message immediately.
-2. Contact DBS Bank directly via their official customer service hotline to inquire about your account status if you have genuine concerns.
-3. Do not provide any personal, financial, or login information to the sender or through the provided link.
-4. Delete the suspicious message to avoid accidentally interacting with it in the future.</t>
+2. Do not click on the provided link or enter any personal or banking information.
+3. Contact your bank directly using the official hotline number found on their official website or on the back of your bank card, to verify the status of your account.
+4. Consider reporting this suspicious message to your local authorities or through official scam reporting channels like ScamShield, if available in your region.
+5. Monitor your bank accounts closely for any unauthorized transactions or suspicious activity.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>1. Access your online banking services only through the official banking application or by typing the bank's official website address directly into your browser.
-2. Be wary of any unsolicited messages or calls that request your passwords, PINs, or OTPs, as legitimate banks will never ask for these details in such a manner.
-3. Enable multi-factor authentication (MFA) on all your banking and online accounts for an added layer of security.
-4. Regularly review your bank statements and account activity for any unauthorized transactions.</t>
+          <t>1. Always access online banking services only through official banking applications or by typing the bank's legitimate website address directly into your browser.
+2. Verify any suspicious messages or calls by contacting your bank through their official customer service channels, not through contact details provided in the suspicious message.
+3. Enable multi-factor authentication and banking transaction notifications on your accounts whenever available, to add an extra layer of security.
+4. Regularly review your bank account activity for any unfamiliar transactions and report them to your bank immediately.
+5. Be wary of any communication that creates undue urgency or threatens negative consequences if immediate action is not taken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="300" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Congratulations! You have been selected for a remote data entry position earning SGD 5,000 per month. No experience is required. Register now at https://easy-work-from-home-jobs.net to secure your position.</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Job Scam</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>91.14%</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>87.64%</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>No - Not required</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>The ScamSense system has assessed this message as a High-risk Job Scam. It appears likely to be a fraudulent offer designed to deceive individuals seeking remote employment opportunities by presenting an unrealistic and unsolicited job offer.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>This message exhibits several characteristics commonly associated with job scams. It offers an unsolicited, high-paying remote position requiring no experience, prompts immediate registration on an external link, and uses an urgent tone, which are all tactics used to lure victims. The Explainable AI identified keywords like 'position', 'remote', 'experience', 'register', and 'congratulations' as contributing to this assessment.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>1. Unsolicited Job Offer with Immediate Selection: The message begins with 'Congratulations! You have been selected...' without any prior application or interview process. This is a common tactic in job scams to create a false sense of opportunity and urgency.
+2. Unrealistic High Income for Minimal Experience: Offering 'SGD 5,000 per month' for a 'remote data entry position' with 'No experience required' is highly unrealistic and designed to attract individuals seeking easy money, which is a key characteristic of fraudulent job offers.
+3. Remote Work and Suspicious Registration Link: The mention of a 'remote data entry position' coupled with an instruction to 'Register now at https://easy-work-from-home-jobs.net' points to common work-from-home scams that often use suspicious or unofficial websites to gather personal information or elicit payments.
+4. Urgency and Lack of Formal Process: The phrase 'secure your position' implies urgency, rushing the user into action without proper vetting, formal interviews, or employment contracts, which legitimate employers typically provide.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>1. Do not click on the provided registration link or interact further with this message. Engaging with such links can lead to phishing attempts or malware.
+2. Never share personal or financial information, such as bank details, identification documents, or login credentials, with unverified recruiters or through suspicious links.
+3. Be extremely wary of any job offer that sounds too good to be true, especially those promising high pay for little effort or no experience.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>1. Block the sender of this message to prevent further scam attempts.
+2. Report the message to your telecommunications provider or the relevant authorities in Singapore, such as the Singapore Police Force (SPF), to help them track and combat such scams.
+3. Delete the message from your device to avoid accidentally interacting with it later.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>1. Always verify job advertisements and recruiter identities through official company websites or recognised recruitment platforms before applying or accepting any offer.
+2. Legitimate employers rarely offer jobs without a formal application process, interviews, or proper assessments. Be suspicious of unsolicited offers or immediate selections.
+3. Never make any payments for job applications, training, or work materials, as legitimate employers do not request fees from job seekers.
+4. Research the employer and the company thoroughly, including checking for reviews or scam reports, before engaging with any job opportunity. Be cautious of companies with generic or newly created online presences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="300" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Your parcel delivery was unsuccessful because the shipping address is incomplete. Please pay a redelivery fee of SGD 2.99 at https://sgparcel-redelivery.com within 24 hours to receive your package.</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Parcel Scam</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>No - Not required</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Based on our analysis, the message you received appears highly likely to be a parcel scam. It exhibits several characteristics commonly used by scammers to trick individuals into making fraudulent payments under the guise of delivery issues.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>The message claims your parcel delivery was unsuccessful due to an incomplete shipping address and demands an urgent redelivery fee of SGD 2.99 to be paid within 24 hours via a provided link (https://sgparcel-redelivery.com). This pattern is highly consistent with parcel scams, where scammers exploit the familiarity of delivery notifications to solicit small, urgent payments or personal information. Legitimate courier companies typically use official channels for such notifications and rarely request fees via suspicious links or with a short deadline. The short timeframe ('within 24 hours') creates a sense of urgency, a common tactic to pressure victims into acting without verifying. The domain name 'sgparcel-redelivery.com' also appears suspicious and is not a standard official courier website, which is a major red flag.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>1. The message is an unsolicited notification claiming a delivery failure for an 'incomplete address.'
+2. It requests an urgent payment (SGD 2.99) for redelivery with a short deadline ('within 24 hours').
+3. It includes a suspicious-looking URL (https://sgparcel-redelivery.com) for making the payment, which is not an official courier website.
+4. The language uses common keywords like 'delivery,' 'package,' and 'parcel' to mimic legitimate communications, a tactic often used in parcel scams.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>1. Do not click on any links provided in unexpected delivery messages.
+2. Do not provide any personal, financial, or account information in response to such messages.
+3. Never make payments based on unexpected or unsolicited delivery notifications.
+4. Verify the status of any expected parcels directly through the official website or mobile application of the courier company, using contact details you find independently, not from the message itself.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>1. Ignore and delete this message immediately.
+2. Report the suspicious message to the relevant authorities, such as through ScamShield if you are in Singapore.
+3. If you have already clicked the link or provided any information, monitor your bank accounts and online accounts for suspicious activity.
+4. If you made a payment or shared banking details, contact your bank immediately to report potential fraud and follow their instructions.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>1. Always verify parcel notifications by checking your recent purchases and expected deliveries directly.
+2. Track parcels only through the courier company's official website or mobile application.
+3. Be cautious of requests for unexpected delivery fees, especially if they come with a sense of urgency.
+4. Before entering any payment information, carefully inspect website addresses to ensure they are legitimate.
+5. Never provide passwords, One-Time Passwords (OTPs), or banking credentials through delivery websites unless you are absolutely certain of their legitimacy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="300" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SingPost is delivering your parcel CNSGS005229637 by today. Please ensure someone is available to receive it. If you are not at home, it will be delivered to a safe place near your doorstep.</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Legitimate</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>48.88%</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>25.48%</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Yes - 3/4 models agreed (75.00%)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Based on our analysis, the message appears likely to be a legitimate parcel delivery notification from SingPost. It provides standard delivery information without significant warning signs commonly associated with scams.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>The message appears legitimate because it describes a routine parcel delivery update from a named courier, SingPost, including a tracking number (CNSGS005229637) and practical instructions for receiving the parcel, such as ensuring someone is available or mentioning delivery to a safe place. This format is consistent with normal service notifications from genuine delivery companies and does not contain unusual requests for payment, sensitive personal details, or suspicious links.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>No scam indicators were identified because this message appears likely to be legitimate.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1. Even though this message appears legitimate, it's always a good practice to exercise caution. If you were not expecting a parcel, or if any delivery message seems unusual, always independently verify its authenticity.
+2. To be absolutely certain, cross-check the delivery status directly on the official SingPost website or app using the provided tracking number (CNSGS005229637), rather than relying solely on links within the message.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>1. Independently verify the parcel's status by visiting SingPost's official website or using their official mobile application and entering the tracking number provided in the message.
+2. Do not click on any links in the message if you are uncertain about its legitimacy, especially if you did not initiate a delivery or purchase recently.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>1. Always track parcels only through the courier company's official website or mobile application.
+2. Be cautious of unsolicited delivery messages, even if they appear genuine, and confirm unexpected notifications with the sender or retailer.
+3. Never provide passwords, One-Time Passwords (OTPs), or banking credentials through unverified delivery websites or links.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M2"/>
+  <autoFilter ref="A1:M5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>